<commit_message>
Regen: stage R_materials_1 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research_materials/03_results/length_control.xlsx
+++ b/research_materials/03_results/length_control.xlsx
@@ -459,7 +459,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Built: 2026-10-06 21:47 by src/build_research_materials.py</t>
+          <t>Built: 2026-10-06 23:35 by src/build_research_materials.py</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -637,33 +637,33 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>test_seen_facts</t>
+          <t>test_trained_exact</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>141.842</v>
+        <v>38.006</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.649</v>
+        <v>0.835</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.523</v>
+        <v>0.696</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0.108</v>
+        <v>0.021</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0.213</v>
+        <v>0.767</v>
       </c>
     </row>
     <row r="5">
@@ -679,28 +679,28 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>base</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>25.115</v>
+        <v>141.842</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0.582</v>
+        <v>0.649</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.316</v>
+        <v>0.523</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>0.105</v>
+        <v>0.108</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>0.263</v>
+        <v>0.213</v>
       </c>
     </row>
     <row r="6">
@@ -711,33 +711,33 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>test_indomain</t>
+          <t>test_seen_facts</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise40</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise base (≤ 40 words)</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>124.168</v>
+        <v>25.115</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.669</v>
+        <v>0.582</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.316</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>0.096</v>
+        <v>0.105</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
     </row>
     <row r="7">
@@ -748,33 +748,33 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>test_indomain</t>
+          <t>test_seen_facts</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>24.988</v>
+        <v>40.412</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.548</v>
+        <v>0.619</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.365</v>
+        <v>0.402</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0.096</v>
+        <v>0.077</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>0.305</v>
+        <v>0.374</v>
       </c>
     </row>
     <row r="8">
@@ -785,7 +785,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>test_heldout_docs</t>
+          <t>test_indomain</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -799,19 +799,19 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>121.7</v>
+        <v>124.168</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.642</v>
+        <v>0.669</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.518</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.096</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0.259</v>
+        <v>0.265</v>
       </c>
     </row>
     <row r="9">
@@ -822,7 +822,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>test_heldout_docs</t>
+          <t>test_indomain</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -836,167 +836,167 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>24.99</v>
+        <v>24.988</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0.547</v>
+        <v>0.548</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.347</v>
+        <v>0.365</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>0.097</v>
+        <v>0.096</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>0.291</v>
+        <v>0.305</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>gemma-4-e4b-it</t>
+          <t>qwen3-8b</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>test_trained_exact</t>
+          <t>test_indomain</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>227.904</v>
+        <v>39.042</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0.702</v>
+        <v>0.494</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.365</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0.073</v>
+        <v>0.09</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>0.173</v>
+        <v>0.331</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>gemma-4-e4b-it</t>
+          <t>qwen3-8b</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>test_trained_exact</t>
+          <t>test_heldout_docs</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>base</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>26.426</v>
+        <v>121.7</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.546</v>
+        <v>0.642</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.316</v>
+        <v>0.518</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.082</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>0.289</v>
+        <v>0.259</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>gemma-4-e4b-it</t>
+          <t>qwen3-8b</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>test_seen_facts</t>
+          <t>test_heldout_docs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise40</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise base (≤ 40 words)</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>237.52</v>
+        <v>24.99</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.668</v>
+        <v>0.547</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0.53</v>
+        <v>0.347</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>0.063</v>
+        <v>0.097</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>0.151</v>
+        <v>0.291</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>gemma-4-e4b-it</t>
+          <t>qwen3-8b</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>test_seen_facts</t>
+          <t>test_heldout_docs</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>26.638</v>
+        <v>38.852</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.595</v>
+        <v>0.431</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>0.303</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>0.077</v>
+        <v>0.102</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0.248</v>
+        <v>0.306</v>
       </c>
     </row>
     <row r="14">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>test_indomain</t>
+          <t>test_trained_exact</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1021,19 +1021,19 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>227.888</v>
+        <v>227.904</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.731</v>
+        <v>0.702</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.574</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>0.078</v>
+        <v>0.073</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>0.177</v>
+        <v>0.173</v>
       </c>
     </row>
     <row r="15">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>test_indomain</t>
+          <t>test_trained_exact</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1058,19 +1058,19 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>26.568</v>
+        <v>26.426</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.595</v>
+        <v>0.546</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.367</v>
+        <v>0.316</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.067</v>
+        <v>0.082</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0.287</v>
+        <v>0.289</v>
       </c>
     </row>
     <row r="16">
@@ -1081,33 +1081,33 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>test_heldout_docs</t>
+          <t>test_trained_exact</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>222.444</v>
+        <v>36.886</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.679</v>
+        <v>0.842</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0.541</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>0.065</v>
+        <v>0.019</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>0.177</v>
+        <v>0.764</v>
       </c>
     </row>
     <row r="17">
@@ -1118,118 +1118,118 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>test_heldout_docs</t>
+          <t>test_seen_facts</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>base</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>27</v>
+        <v>237.52</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.668</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>0.343</v>
+        <v>0.53</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>0.068</v>
+        <v>0.063</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>0.276</v>
+        <v>0.151</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>test_trained_exact</t>
+          <t>test_seen_facts</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise40</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise base (≤ 40 words)</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>222.082</v>
+        <v>26.638</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0.552</v>
+        <v>0.595</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0.517</v>
+        <v>0.303</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>0.1</v>
+        <v>0.077</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0.179</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>test_trained_exact</t>
+          <t>test_seen_facts</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>35.048</v>
+        <v>41.219</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0.478</v>
+        <v>0.613</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>0.369</v>
+        <v>0.435</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>0.117</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>0.324</v>
+        <v>0.393</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>test_seen_facts</t>
+          <t>test_indomain</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1243,30 +1243,30 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>227.853</v>
+        <v>227.888</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0.522</v>
+        <v>0.731</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0.498</v>
+        <v>0.574</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>0.083</v>
+        <v>0.078</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>0.154</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>test_seen_facts</t>
+          <t>test_indomain</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1280,25 +1280,25 @@
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>37.477</v>
+        <v>26.568</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.53</v>
+        <v>0.595</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.356</v>
+        <v>0.367</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>0.115</v>
+        <v>0.067</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>0.265</v>
+        <v>0.287</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1308,71 +1308,71 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ep3</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>QA-only ep3</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>219.658</v>
+        <v>38.538</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0.575</v>
+        <v>0.496</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>0.555</v>
+        <v>0.355</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0.091</v>
+        <v>0.078</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0.182</v>
+        <v>0.324</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>test_indomain</t>
+          <t>test_heldout_docs</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>concise40</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>concise base (≤ 40 words)</t>
+          <t>base</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>37.004</v>
+        <v>222.444</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0.51</v>
+        <v>0.679</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0.418</v>
+        <v>0.541</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>0.102</v>
+        <v>0.065</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0.322</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>llama-3.1-8b-instruct</t>
+          <t>gemma-4-e4b-it</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1382,65 +1382,509 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise40</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>concise base (≤ 40 words)</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
-        <v>212.764</v>
+        <v>27</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0.534</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>0.493</v>
+        <v>0.343</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>0.1</v>
+        <v>0.068</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>0.179</v>
+        <v>0.276</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>gemma-4-e4b-it</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>test_heldout_docs</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ep3</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>QA-only ep3</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>38.078</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>0.301</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>llama-3.1-8b-instruct</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>test_trained_exact</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>222.082</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>0.179</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>test_trained_exact</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>concise40</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>concise base (≤ 40 words)</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>35.048</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>0.324</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>test_trained_exact</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>ep2</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>QA-only ep2</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>38.306</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>0.823</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>test_seen_facts</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>227.853</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>0.498</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0.083</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>0.154</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>test_seen_facts</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>concise40</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>concise base (≤ 40 words)</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>37.477</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>0.265</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>test_seen_facts</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>ep2</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>QA-only ep2</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>42.566</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0.719</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>0.544</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0.544</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>test_indomain</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>219.658</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0.091</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>0.182</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>test_indomain</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>concise40</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>concise base (≤ 40 words)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>37.004</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>0.322</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>test_indomain</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>ep2</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>QA-only ep2</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>39.946</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0.501</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>test_heldout_docs</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>212.764</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>0.534</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>0.493</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>0.179</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>test_heldout_docs</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>concise40</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>concise base (≤ 40 words)</t>
         </is>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E36" s="3" t="n">
         <v>35.842</v>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="F36" s="3" t="n">
         <v>0.506</v>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="G36" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="H25" s="3" t="n">
+      <c r="H36" s="3" t="n">
         <v>0.102</v>
       </c>
-      <c r="I25" s="3" t="n">
+      <c r="I36" s="3" t="n">
         <v>0.311</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>llama-3.1-8b-instruct</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>test_heldout_docs</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>ep2</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>QA-only ep2</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>41.284</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>0.312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>